<commit_message>
Update CPCA Calculator to 3-tab layout
</commit_message>
<xml_diff>
--- a/MFDS 1일 섭취허용량.xlsx
+++ b/MFDS 1일 섭취허용량.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a624188ccc7a469/바탕 화면/CPCA 계산기/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a624188ccc7a469/바탕 화면/nitrosamines-AI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_769BC176CB385EDFDA183B0CA155A9EDADF59F72" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF0B93A6-4A2C-4D4A-8BC2-57AF8B2FBE69}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_769BC176CB385EDFDA183B0CA155A9EDADF59F72" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45B4DB18-BB0D-4230-AD37-4B608B7537B8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="26690" yWindow="5180" windowWidth="14400" windowHeight="8240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -2529,18 +2529,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:I158"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="2" max="2" width="36.33203125" customWidth="1"/>
+    <col min="2" max="2" width="36.3125" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" customWidth="1"/>
     <col min="4" max="4" width="47.75" customWidth="1"/>
     <col min="5" max="5" width="23.5" customWidth="1"/>
-    <col min="8" max="8" width="27.58203125" customWidth="1"/>
+    <col min="8" max="8" width="27.5625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2569,7 +2568,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="187" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" ht="185.65" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2592,7 +2591,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -2618,7 +2617,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2644,7 +2643,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -2667,7 +2666,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -2693,7 +2692,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -2716,7 +2715,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="289" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:9" ht="270" x14ac:dyDescent="0.6">
       <c r="A8" t="s">
         <v>41</v>
       </c>
@@ -2742,7 +2741,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -2768,7 +2767,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -2791,7 +2790,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2817,7 +2816,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A12" t="s">
         <v>62</v>
       </c>
@@ -2840,7 +2839,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -2863,7 +2862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -2886,7 +2885,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -2909,7 +2908,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -2932,7 +2931,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A17" t="s">
         <v>83</v>
       </c>
@@ -2955,7 +2954,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A18" t="s">
         <v>86</v>
       </c>
@@ -2978,7 +2977,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="119" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:9" ht="118.15" x14ac:dyDescent="0.6">
       <c r="A19" t="s">
         <v>90</v>
       </c>
@@ -3001,7 +3000,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -3024,7 +3023,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A21" t="s">
         <v>97</v>
       </c>
@@ -3050,7 +3049,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A22" t="s">
         <v>102</v>
       </c>
@@ -3073,7 +3072,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A23" t="s">
         <v>106</v>
       </c>
@@ -3096,7 +3095,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A24" t="s">
         <v>111</v>
       </c>
@@ -3119,7 +3118,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A25" t="s">
         <v>118</v>
       </c>
@@ -3145,7 +3144,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A26" t="s">
         <v>124</v>
       </c>
@@ -3168,7 +3167,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A27" t="s">
         <v>128</v>
       </c>
@@ -3194,7 +3193,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A28" t="s">
         <v>133</v>
       </c>
@@ -3217,7 +3216,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A29" t="s">
         <v>138</v>
       </c>
@@ -3240,7 +3239,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A30" t="s">
         <v>142</v>
       </c>
@@ -3263,7 +3262,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A31" t="s">
         <v>146</v>
       </c>
@@ -3286,7 +3285,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A32" t="s">
         <v>150</v>
       </c>
@@ -3309,7 +3308,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A33" t="s">
         <v>155</v>
       </c>
@@ -3332,7 +3331,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A34" t="s">
         <v>159</v>
       </c>
@@ -3355,7 +3354,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A35" t="s">
         <v>163</v>
       </c>
@@ -3381,7 +3380,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A36" t="s">
         <v>168</v>
       </c>
@@ -3407,7 +3406,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="102" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:9" ht="101.25" x14ac:dyDescent="0.6">
       <c r="A37" t="s">
         <v>175</v>
       </c>
@@ -3433,7 +3432,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A38" t="s">
         <v>181</v>
       </c>
@@ -3459,7 +3458,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A39" t="s">
         <v>186</v>
       </c>
@@ -3482,7 +3481,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A40" t="s">
         <v>190</v>
       </c>
@@ -3505,7 +3504,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A41" t="s">
         <v>195</v>
       </c>
@@ -3528,7 +3527,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A42" t="s">
         <v>199</v>
       </c>
@@ -3554,7 +3553,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A43" t="s">
         <v>204</v>
       </c>
@@ -3577,7 +3576,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A44" t="s">
         <v>207</v>
       </c>
@@ -3603,7 +3602,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A45" t="s">
         <v>212</v>
       </c>
@@ -3629,7 +3628,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A46" t="s">
         <v>216</v>
       </c>
@@ -3655,7 +3654,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="102" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:9" ht="101.25" x14ac:dyDescent="0.6">
       <c r="A47" t="s">
         <v>221</v>
       </c>
@@ -3678,7 +3677,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A48" t="s">
         <v>225</v>
       </c>
@@ -3701,7 +3700,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A49" t="s">
         <v>229</v>
       </c>
@@ -3724,7 +3723,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A50" t="s">
         <v>233</v>
       </c>
@@ -3747,7 +3746,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A51" t="s">
         <v>237</v>
       </c>
@@ -3770,7 +3769,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A52" t="s">
         <v>242</v>
       </c>
@@ -3793,7 +3792,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A53" t="s">
         <v>246</v>
       </c>
@@ -3819,7 +3818,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A54" t="s">
         <v>250</v>
       </c>
@@ -3845,7 +3844,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="221" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:9" ht="202.5" x14ac:dyDescent="0.6">
       <c r="A55" t="s">
         <v>255</v>
       </c>
@@ -3868,7 +3867,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A56" t="s">
         <v>259</v>
       </c>
@@ -3894,7 +3893,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A57" t="s">
         <v>264</v>
       </c>
@@ -3920,7 +3919,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A58" t="s">
         <v>269</v>
       </c>
@@ -3946,7 +3945,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A59" t="s">
         <v>52</v>
       </c>
@@ -3969,7 +3968,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A60" t="s">
         <v>276</v>
       </c>
@@ -3992,7 +3991,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A61" t="s">
         <v>280</v>
       </c>
@@ -4018,7 +4017,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A62" t="s">
         <v>285</v>
       </c>
@@ -4041,7 +4040,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A63" t="s">
         <v>18</v>
       </c>
@@ -4064,7 +4063,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A64" t="s">
         <v>293</v>
       </c>
@@ -4087,7 +4086,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A65" t="s">
         <v>297</v>
       </c>
@@ -4110,7 +4109,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A66" t="s">
         <v>301</v>
       </c>
@@ -4133,7 +4132,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A67" t="s">
         <v>305</v>
       </c>
@@ -4159,7 +4158,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A68" t="s">
         <v>310</v>
       </c>
@@ -4182,7 +4181,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A69" t="s">
         <v>314</v>
       </c>
@@ -4205,7 +4204,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A70" t="s">
         <v>318</v>
       </c>
@@ -4231,7 +4230,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A71" t="s">
         <v>323</v>
       </c>
@@ -4254,7 +4253,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A72" t="s">
         <v>327</v>
       </c>
@@ -4277,7 +4276,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A73" t="s">
         <v>330</v>
       </c>
@@ -4300,7 +4299,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A74" t="s">
         <v>334</v>
       </c>
@@ -4326,7 +4325,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A75" t="s">
         <v>338</v>
       </c>
@@ -4349,7 +4348,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A76" t="s">
         <v>342</v>
       </c>
@@ -4375,7 +4374,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A77" t="s">
         <v>347</v>
       </c>
@@ -4398,7 +4397,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A78" t="s">
         <v>351</v>
       </c>
@@ -4424,7 +4423,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A79" t="s">
         <v>357</v>
       </c>
@@ -4450,7 +4449,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A80" t="s">
         <v>361</v>
       </c>
@@ -4473,7 +4472,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A81" t="s">
         <v>365</v>
       </c>
@@ -4499,7 +4498,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A82" t="s">
         <v>371</v>
       </c>
@@ -4525,7 +4524,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A83" t="s">
         <v>375</v>
       </c>
@@ -4548,7 +4547,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A84" t="s">
         <v>379</v>
       </c>
@@ -4574,7 +4573,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A85" t="s">
         <v>384</v>
       </c>
@@ -4597,7 +4596,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A86" t="s">
         <v>388</v>
       </c>
@@ -4623,7 +4622,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A87" t="s">
         <v>393</v>
       </c>
@@ -4646,7 +4645,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A88" t="s">
         <v>397</v>
       </c>
@@ -4669,7 +4668,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A89" t="s">
         <v>401</v>
       </c>
@@ -4692,7 +4691,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A90" t="s">
         <v>405</v>
       </c>
@@ -4715,7 +4714,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="119" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:9" ht="118.15" x14ac:dyDescent="0.6">
       <c r="A91" t="s">
         <v>409</v>
       </c>
@@ -4738,7 +4737,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A92" t="s">
         <v>412</v>
       </c>
@@ -4764,7 +4763,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A93" t="s">
         <v>417</v>
       </c>
@@ -4790,7 +4789,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A94" t="s">
         <v>422</v>
       </c>
@@ -4816,7 +4815,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A95" t="s">
         <v>427</v>
       </c>
@@ -4839,7 +4838,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A96" t="s">
         <v>431</v>
       </c>
@@ -4865,7 +4864,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A97" t="s">
         <v>435</v>
       </c>
@@ -4888,7 +4887,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A98" t="s">
         <v>439</v>
       </c>
@@ -4914,7 +4913,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A99" t="s">
         <v>444</v>
       </c>
@@ -4937,7 +4936,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A100" t="s">
         <v>448</v>
       </c>
@@ -4960,7 +4959,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A101" t="s">
         <v>452</v>
       </c>
@@ -4983,7 +4982,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A102" t="s">
         <v>455</v>
       </c>
@@ -5009,7 +5008,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A103" t="s">
         <v>461</v>
       </c>
@@ -5032,7 +5031,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A104" t="s">
         <v>465</v>
       </c>
@@ -5055,7 +5054,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A105" t="s">
         <v>469</v>
       </c>
@@ -5078,7 +5077,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A106" t="s">
         <v>472</v>
       </c>
@@ -5101,7 +5100,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A107" t="s">
         <v>475</v>
       </c>
@@ -5124,7 +5123,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A108" t="s">
         <v>479</v>
       </c>
@@ -5147,7 +5146,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A109" t="s">
         <v>482</v>
       </c>
@@ -5173,7 +5172,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A110" t="s">
         <v>487</v>
       </c>
@@ -5196,7 +5195,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A111" t="s">
         <v>490</v>
       </c>
@@ -5222,7 +5221,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="102" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:9" ht="101.25" x14ac:dyDescent="0.6">
       <c r="A112" t="s">
         <v>495</v>
       </c>
@@ -5245,7 +5244,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A113" t="s">
         <v>499</v>
       </c>
@@ -5268,7 +5267,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A114" t="s">
         <v>503</v>
       </c>
@@ -5291,7 +5290,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A115" t="s">
         <v>507</v>
       </c>
@@ -5314,7 +5313,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A116" t="s">
         <v>511</v>
       </c>
@@ -5337,7 +5336,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A117" t="s">
         <v>515</v>
       </c>
@@ -5360,7 +5359,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A118" t="s">
         <v>519</v>
       </c>
@@ -5383,7 +5382,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A119" t="s">
         <v>523</v>
       </c>
@@ -5406,7 +5405,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A120" t="s">
         <v>526</v>
       </c>
@@ -5432,7 +5431,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A121" t="s">
         <v>530</v>
       </c>
@@ -5455,7 +5454,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A122" t="s">
         <v>533</v>
       </c>
@@ -5478,7 +5477,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A123" t="s">
         <v>536</v>
       </c>
@@ -5501,7 +5500,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A124" t="s">
         <v>540</v>
       </c>
@@ -5524,7 +5523,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A125" t="s">
         <v>543</v>
       </c>
@@ -5547,7 +5546,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A126" t="s">
         <v>547</v>
       </c>
@@ -5573,7 +5572,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A127" t="s">
         <v>552</v>
       </c>
@@ -5599,7 +5598,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A128" t="s">
         <v>557</v>
       </c>
@@ -5625,7 +5624,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A129" t="s">
         <v>562</v>
       </c>
@@ -5648,7 +5647,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A130" t="s">
         <v>566</v>
       </c>
@@ -5671,7 +5670,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A131" t="s">
         <v>570</v>
       </c>
@@ -5697,7 +5696,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A132" t="s">
         <v>575</v>
       </c>
@@ -5723,7 +5722,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A133" t="s">
         <v>580</v>
       </c>
@@ -5746,7 +5745,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A134" t="s">
         <v>584</v>
       </c>
@@ -5769,7 +5768,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:9" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A135" t="s">
         <v>588</v>
       </c>
@@ -5792,7 +5791,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A136" t="s">
         <v>592</v>
       </c>
@@ -5815,7 +5814,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A137" t="s">
         <v>596</v>
       </c>
@@ -5838,7 +5837,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A138" t="s">
         <v>600</v>
       </c>
@@ -5861,7 +5860,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A139" t="s">
         <v>604</v>
       </c>
@@ -5884,7 +5883,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A140" t="s">
         <v>608</v>
       </c>
@@ -5910,7 +5909,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A141" t="s">
         <v>613</v>
       </c>
@@ -5933,7 +5932,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="85" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A142" t="s">
         <v>617</v>
       </c>
@@ -5956,7 +5955,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A143" t="s">
         <v>621</v>
       </c>
@@ -5982,7 +5981,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="51" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:9" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A144" t="s">
         <v>627</v>
       </c>
@@ -6008,7 +6007,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A145" t="s">
         <v>632</v>
       </c>
@@ -6034,7 +6033,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="68" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:9" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A146" t="s">
         <v>638</v>
       </c>
@@ -6057,7 +6056,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A147" t="s">
         <v>642</v>
       </c>
@@ -6083,7 +6082,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A148" t="s">
         <v>646</v>
       </c>
@@ -6109,7 +6108,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="34" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:9" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A149" t="s">
         <v>650</v>
       </c>
@@ -6135,7 +6134,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A150" t="s">
         <v>654</v>
       </c>
@@ -6161,7 +6160,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A151" t="s">
         <v>658</v>
       </c>
@@ -6187,7 +6186,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A152" t="s">
         <v>662</v>
       </c>
@@ -6210,7 +6209,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A153" t="s">
         <v>666</v>
       </c>
@@ -6233,7 +6232,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A154" t="s">
         <v>31</v>
       </c>
@@ -6256,7 +6255,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A155" t="s">
         <v>12</v>
       </c>
@@ -6282,7 +6281,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A156" t="s">
         <v>24</v>
       </c>
@@ -6308,7 +6307,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A157" t="s">
         <v>51</v>
       </c>
@@ -6331,7 +6330,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A158" t="s">
         <v>56</v>
       </c>
@@ -6355,13 +6354,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I158" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="5">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I158" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>